<commit_message>
Terraform, Databricks, and Snowflake Gold Layer. Working on dbt.
</commit_message>
<xml_diff>
--- a/data/Vancouver-Housing-Data.xlsx
+++ b/data/Vancouver-Housing-Data.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alanhu/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alanhu/Desktop/Vancouver Housing Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CEC7797-6D9E-E84D-95B6-3CC70E60BF5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{081250C2-E421-054A-B971-90CAADA853C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14520" yWindow="0" windowWidth="14280" windowHeight="18000" xr2:uid="{94874A01-71C6-544D-8A61-0EE0FAE343D3}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{94874A01-71C6-544D-8A61-0EE0FAE343D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="30">
   <si>
     <t>Neighbourhood</t>
   </si>
@@ -111,12 +111,31 @@
   </si>
   <si>
     <t>Killarney</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Townhouses</t>
+  </si>
+  <si>
+    <t>Condo</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Detached</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="5" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="167" formatCode="mmm\ yyyy"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -146,13 +165,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="5" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <numFmt numFmtId="167" formatCode="mmm\ yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="9" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\)"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -163,6 +191,19 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61FF07C3-FA9E-6F40-9658-301C00BA2DA4}" name="Table1" displayName="Table1" ref="A1:D67" totalsRowShown="0">
+  <autoFilter ref="A1:D67" xr:uid="{61FF07C3-FA9E-6F40-9658-301C00BA2DA4}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{9E2F1382-D097-2842-BD73-809F795F8A41}" name="Neighbourhood"/>
+    <tableColumn id="2" xr3:uid="{0D036537-D78E-3246-934D-185F6EE0068A}" name="Type of Property"/>
+    <tableColumn id="4" xr3:uid="{3AB14105-3CBE-7847-B478-4691EC03BE33}" name="Date" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{F2DCEEB6-B8C5-684F-A6C1-CA4F4561592A}" name="Price" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -482,135 +523,925 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F61AE828-A24F-E648-ABFE-E7CE3A96365B}">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.6640625" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1134200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D4" s="1">
+        <v>633100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1099100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D7" s="1">
+        <v>639400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1488100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D9" s="1">
+        <v>901400</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D10" s="1">
+        <v>667900</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1697800</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D12" s="1">
+        <v>1257000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D13" s="1">
+        <v>601500</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D14" s="1">
+        <v>1592300</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D16" s="1">
+        <v>501500</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="B20" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D20" s="1">
+        <v>2548600</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D21" s="1">
+        <v>1268900</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D22" s="1">
+        <v>700800</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="B23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D24" s="1">
+        <v>989600</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D25" s="1">
+        <v>770100</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="B26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D26" s="1">
+        <f xml:space="preserve"> (2098400 + 1709200)/2</f>
+        <v>1903800</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D27" s="1">
+        <f xml:space="preserve"> (1207800 + 1072400) / 2</f>
+        <v>1140100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D28" s="1">
+        <f xml:space="preserve"> (660800 + 673900) / 2</f>
+        <v>667350</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="B29" t="s">
+        <v>29</v>
+      </c>
+      <c r="C29" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D29" s="1">
+        <v>2672000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
+        <v>26</v>
+      </c>
+      <c r="C30" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" t="s">
+        <v>27</v>
+      </c>
+      <c r="C31" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D31" s="1">
+        <v>951300</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="B32" t="s">
+        <v>29</v>
+      </c>
+      <c r="C32" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D32" s="1">
+        <v>3260200</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>6</v>
+      </c>
+      <c r="B33" t="s">
+        <v>26</v>
+      </c>
+      <c r="C33" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C34" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="B35" t="s">
+        <v>29</v>
+      </c>
+      <c r="C35" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D35" s="1">
+        <v>4133900</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>15</v>
+      </c>
+      <c r="B36" t="s">
+        <v>26</v>
+      </c>
+      <c r="C36" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>15</v>
+      </c>
+      <c r="B37" t="s">
+        <v>27</v>
+      </c>
+      <c r="C37" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D37" s="1">
+        <v>1018700</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="B38" t="s">
+        <v>29</v>
+      </c>
+      <c r="C38" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D38" s="1">
+        <v>4160200</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>16</v>
+      </c>
+      <c r="B39" t="s">
+        <v>26</v>
+      </c>
+      <c r="C39" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D39" s="1">
+        <v>1556400</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>16</v>
+      </c>
+      <c r="B40" t="s">
+        <v>27</v>
+      </c>
+      <c r="C40" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D40" s="1">
+        <v>1017700</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="B41" t="s">
+        <v>29</v>
+      </c>
+      <c r="C41" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" t="s">
+        <v>26</v>
+      </c>
+      <c r="C42" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>17</v>
+      </c>
+      <c r="B43" t="s">
+        <v>27</v>
+      </c>
+      <c r="C43" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="B44" t="s">
+        <v>29</v>
+      </c>
+      <c r="C44" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>18</v>
+      </c>
+      <c r="B45" t="s">
+        <v>26</v>
+      </c>
+      <c r="C45" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>18</v>
+      </c>
+      <c r="B46" t="s">
+        <v>27</v>
+      </c>
+      <c r="C46" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="B47" t="s">
+        <v>29</v>
+      </c>
+      <c r="C47" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D47" s="1">
+        <v>1607600</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>19</v>
+      </c>
+      <c r="B48" t="s">
+        <v>26</v>
+      </c>
+      <c r="C48" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D48" s="1">
+        <v>900600</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>19</v>
+      </c>
+      <c r="B49" t="s">
+        <v>27</v>
+      </c>
+      <c r="C49" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D49" s="1">
+        <v>677700</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="B50" t="s">
+        <v>29</v>
+      </c>
+      <c r="C50" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D50" s="1">
+        <v>2981000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>7</v>
+      </c>
+      <c r="B51" t="s">
+        <v>26</v>
+      </c>
+      <c r="C51" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D51" s="1">
+        <v>1663000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>7</v>
+      </c>
+      <c r="B52" t="s">
+        <v>27</v>
+      </c>
+      <c r="C52" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D52" s="1">
+        <v>974200</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="B53" t="s">
+        <v>29</v>
+      </c>
+      <c r="C53" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D53" s="1">
+        <v>3364500</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>20</v>
+      </c>
+      <c r="B54" t="s">
+        <v>26</v>
+      </c>
+      <c r="C54" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D54" s="1">
+        <v>1635800</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>20</v>
+      </c>
+      <c r="B55" t="s">
+        <v>27</v>
+      </c>
+      <c r="C55" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D55" s="1">
+        <v>997900</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="B56" t="s">
+        <v>29</v>
+      </c>
+      <c r="C56" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D56" s="1">
+        <v>2134900</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>21</v>
+      </c>
+      <c r="B57" t="s">
+        <v>26</v>
+      </c>
+      <c r="C57" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D57" s="1">
+        <v>1575700</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>21</v>
+      </c>
+      <c r="B58" t="s">
+        <v>27</v>
+      </c>
+      <c r="C58" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D58" s="1">
+        <v>683800</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="B59" t="s">
+        <v>29</v>
+      </c>
+      <c r="C59" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>22</v>
+      </c>
+      <c r="B60" t="s">
+        <v>26</v>
+      </c>
+      <c r="C60" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>22</v>
+      </c>
+      <c r="B61" t="s">
+        <v>27</v>
+      </c>
+      <c r="C61" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+      <c r="B62" t="s">
+        <v>29</v>
+      </c>
+      <c r="C62" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D62" s="1">
+        <v>1662400</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>23</v>
+      </c>
+      <c r="B63" t="s">
+        <v>26</v>
+      </c>
+      <c r="C63" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D63" s="1">
+        <v>1153600</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>23</v>
+      </c>
+      <c r="B64" t="s">
+        <v>27</v>
+      </c>
+      <c r="C64" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D64" s="1">
+        <v>692200</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
         <v>24</v>
+      </c>
+      <c r="B65" t="s">
+        <v>29</v>
+      </c>
+      <c r="C65" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D65" s="1">
+        <v>1756900</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>24</v>
+      </c>
+      <c r="B66" t="s">
+        <v>26</v>
+      </c>
+      <c r="C66" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D66" s="1">
+        <v>842500</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>24</v>
+      </c>
+      <c r="B67" t="s">
+        <v>27</v>
+      </c>
+      <c r="C67" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D67" s="1">
+        <v>538500</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>